<commit_message>
changes to Y and rho for the plants
</commit_message>
<xml_diff>
--- a/experiments/batch_results_pepper0/results_summary.xlsx
+++ b/experiments/batch_results_pepper0/results_summary.xlsx
@@ -592,19 +592,19 @@
         <v>0.7</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6000000000000001</v>
+        <v>0.7002548307756539</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6000000000000001</v>
+        <v>0.7002547179550054</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6000000000000001</v>
+        <v>0.7002545828071589</v>
       </c>
       <c r="E2" t="n">
-        <v>0.6000000000000001</v>
+        <v>0.7002544190357363</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6000000000000001</v>
+        <v>0.700254220606405</v>
       </c>
     </row>
     <row r="3">
@@ -612,19 +612,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>1.000151968891649</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>1.000150013027004</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>1.00014809371153</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>1.000146223334927</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>1.000144414094734</v>
       </c>
     </row>
     <row r="4">
@@ -632,19 +632,19 @@
         <v>1.3</v>
       </c>
       <c r="B4" t="n">
-        <v>1.2</v>
+        <v>1.300063544338489</v>
       </c>
       <c r="C4" t="n">
-        <v>1.2</v>
+        <v>1.300063531892054</v>
       </c>
       <c r="D4" t="n">
-        <v>1.2</v>
+        <v>1.300063501899238</v>
       </c>
       <c r="E4" t="n">
-        <v>1.2</v>
+        <v>1.300063450224354</v>
       </c>
       <c r="F4" t="n">
-        <v>1.2</v>
+        <v>1.300063373761627</v>
       </c>
     </row>
     <row r="5">
@@ -652,19 +652,19 @@
         <v>1.6</v>
       </c>
       <c r="B5" t="n">
-        <v>1.6</v>
+        <v>1.600035652336454</v>
       </c>
       <c r="C5" t="n">
-        <v>1.6</v>
+        <v>1.600034965047131</v>
       </c>
       <c r="D5" t="n">
-        <v>1.6</v>
+        <v>1.600034315816131</v>
       </c>
       <c r="E5" t="n">
-        <v>1.6</v>
+        <v>1.600033718024373</v>
       </c>
       <c r="F5" t="n">
-        <v>1.6</v>
+        <v>1.600033184969037</v>
       </c>
     </row>
     <row r="6">
@@ -672,19 +672,19 @@
         <v>1.9</v>
       </c>
       <c r="B6" t="n">
-        <v>1.8</v>
+        <v>1.900021300074581</v>
       </c>
       <c r="C6" t="n">
-        <v>1.8</v>
+        <v>1.90002130159797</v>
       </c>
       <c r="D6" t="n">
-        <v>1.8</v>
+        <v>1.900021293869876</v>
       </c>
       <c r="E6" t="n">
-        <v>1.8</v>
+        <v>1.90002127741654</v>
       </c>
       <c r="F6" t="n">
-        <v>1.8</v>
+        <v>1.900021255675643</v>
       </c>
     </row>
   </sheetData>

</xml_diff>